<commit_message>
Aktualizovat data vinné karty z ERP (2026-10-09)
</commit_message>
<xml_diff>
--- a/data/Enoteka_pozice.xlsx
+++ b/data/Enoteka_pozice.xlsx
@@ -1875,7 +1875,7 @@
     <t>ZNO.0472</t>
   </si>
   <si>
-    <t>22,6</t>
+    <t>14,4</t>
   </si>
   <si>
     <t>Je krásný, typický, odrůdový, zaujme hned na první přivonění. Najdete v něm květ bezu, zralý angrešt nebo černý rybíz. Chuť je bohatá, čistá a harmonická, s tóny manga, liči nebo kompotovaného ananasu. Milovníky Hibernalu toto víno jistě potěší.</t>
@@ -7517,7 +7517,7 @@
         <v>100</v>
       </c>
       <c r="D82" t="s">
-        <v>152</v>
+        <v>24</v>
       </c>
       <c r="E82" t="n">
         <v>2025.0</v>
@@ -7925,7 +7925,7 @@
         <v>489</v>
       </c>
       <c r="D88" t="s">
-        <v>152</v>
+        <v>24</v>
       </c>
       <c r="E88" t="n">
         <v>2024.0</v>
@@ -8171,7 +8171,7 @@
         <v>286</v>
       </c>
       <c r="R91" t="s">
-        <v>152</v>
+        <v>374</v>
       </c>
       <c r="S91" t="s">
         <v>33</v>
@@ -9829,7 +9829,7 @@
         <v>75</v>
       </c>
       <c r="D116" t="s">
-        <v>152</v>
+        <v>220</v>
       </c>
       <c r="E116" t="n">
         <v>2025.0</v>

</xml_diff>

<commit_message>
Aktualizovat data vinné karty z ERP (2026-10-13)
</commit_message>
<xml_diff>
--- a/data/Enoteka_pozice.xlsx
+++ b/data/Enoteka_pozice.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1706" uniqueCount="645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1706" uniqueCount="647">
   <si>
     <t>Je_v_ENO</t>
   </si>
@@ -1845,13 +1845,19 @@
     <t>YRUMNUQ3BL</t>
   </si>
   <si>
-    <t>VAN.0136</t>
-  </si>
-  <si>
-    <t>Polosuché bílé víno odrůdy Sauvignon ročníku 2024 z vinařství Jana Vaňka, zatříděné do apelačního systému VOC Znojmo v dubnu 2025. Typický znojemský Sauvignon má výrazný aromatický profil plný opulentních tónů černého rybízu, angreštu a broskví. Ovocné tóny přecházejí také do chuti, kde jsou doplněny tóny citrusů, které přecházejí v příjemně minerální závěr. Nezbytností je svěží kyselinka, která je pevnou páteří vína.</t>
-  </si>
-  <si>
-    <t>YRKNTUJLS3</t>
+    <t xml:space="preserve">Muškát Moravský </t>
+  </si>
+  <si>
+    <t>VAN.0132</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muškát moravský </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aromatické suché víno odrůdy Muškát moravský z rodinného Vinařství Vaněk z Vrbovce. </t>
+  </si>
+  <si>
+    <t>YRKLYQTZ7F</t>
   </si>
   <si>
     <t>VIH.0261</t>
@@ -9622,16 +9628,16 @@
         <v>112.0</v>
       </c>
       <c r="C113" t="s">
-        <v>246</v>
+        <v>609</v>
       </c>
       <c r="D113" t="s">
-        <v>220</v>
+        <v>24</v>
       </c>
       <c r="E113" t="n">
         <v>2024.0</v>
       </c>
       <c r="F113" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="G113" t="s">
         <v>247</v>
@@ -9652,34 +9658,34 @@
         <v>70.0</v>
       </c>
       <c r="M113" t="n">
-        <v>231.0</v>
+        <v>192.99</v>
       </c>
       <c r="N113" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="O113" t="s">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="P113" t="s">
-        <v>482</v>
+        <v>173</v>
       </c>
       <c r="Q113" t="s">
-        <v>501</v>
+        <v>65</v>
       </c>
       <c r="R113" t="s">
         <v>32</v>
       </c>
       <c r="S113" t="s">
-        <v>43</v>
+        <v>311</v>
       </c>
       <c r="T113" t="s">
-        <v>246</v>
+        <v>611</v>
       </c>
       <c r="U113" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="V113" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
     </row>
     <row r="114">
@@ -9723,7 +9729,7 @@
         <v>189.0</v>
       </c>
       <c r="N114" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="O114" t="n">
         <v>12.0</v>
@@ -9744,10 +9750,10 @@
         <v>204</v>
       </c>
       <c r="U114" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="V114" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
     </row>
     <row r="115">
@@ -9791,13 +9797,13 @@
         <v>199.0</v>
       </c>
       <c r="N115" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="O115" t="s">
         <v>40</v>
       </c>
       <c r="P115" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="Q115" t="s">
         <v>42</v>
@@ -9815,7 +9821,7 @@
         <v>152</v>
       </c>
       <c r="V115" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="116">
@@ -9859,13 +9865,13 @@
         <v>180.0</v>
       </c>
       <c r="N116" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="O116" t="s">
         <v>78</v>
       </c>
       <c r="P116" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="Q116" t="s">
         <v>99</v>
@@ -9880,10 +9886,10 @@
         <v>75</v>
       </c>
       <c r="U116" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="V116" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
     </row>
     <row r="117">
@@ -9894,7 +9900,7 @@
         <v>116.0</v>
       </c>
       <c r="C117" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="D117" t="s">
         <v>220</v>
@@ -9927,7 +9933,7 @@
         <v>180.0</v>
       </c>
       <c r="N117" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="O117" t="s">
         <v>40</v>
@@ -9945,13 +9951,13 @@
         <v>33</v>
       </c>
       <c r="T117" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="U117" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="V117" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
     </row>
     <row r="118">
@@ -9962,7 +9968,7 @@
         <v>117.0</v>
       </c>
       <c r="C118" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="D118" t="s">
         <v>24</v>
@@ -9995,7 +10001,7 @@
         <v>150.0</v>
       </c>
       <c r="N118" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="O118" t="n">
         <v>12.0</v>
@@ -10010,16 +10016,16 @@
         <v>32</v>
       </c>
       <c r="S118" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="T118" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="U118" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="V118" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
     </row>
     <row r="119">
@@ -10030,7 +10036,7 @@
         <v>118.0</v>
       </c>
       <c r="C119" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="D119" t="s">
         <v>24</v>
@@ -10063,13 +10069,13 @@
         <v>182.0</v>
       </c>
       <c r="N119" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="O119" t="n">
         <v>13.0</v>
       </c>
       <c r="P119" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="Q119" t="s">
         <v>114</v>
@@ -10078,16 +10084,16 @@
         <v>32</v>
       </c>
       <c r="S119" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="T119" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="U119" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="V119" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
     </row>
     <row r="120">
@@ -10098,7 +10104,7 @@
         <v>119.0</v>
       </c>
       <c r="C120" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="D120" t="s">
         <v>24</v>
@@ -10131,7 +10137,7 @@
         <v>175.0</v>
       </c>
       <c r="N120" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="O120" t="n">
         <v>12.0</v>
@@ -10149,13 +10155,13 @@
         <v>397</v>
       </c>
       <c r="T120" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="U120" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="V120" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
     </row>
     <row r="121">
@@ -10166,7 +10172,7 @@
         <v>120.0</v>
       </c>
       <c r="C121" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="D121" t="s">
         <v>24</v>
@@ -10199,7 +10205,7 @@
         <v>160.0</v>
       </c>
       <c r="N121" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="O121" t="n">
         <v>14.0</v>
@@ -10217,13 +10223,13 @@
         <v>406</v>
       </c>
       <c r="T121" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="U121" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="V121" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aktualizovat data vinné karty z ERP (2026-10-21)
</commit_message>
<xml_diff>
--- a/data/Enoteka_pozice.xlsx
+++ b/data/Enoteka_pozice.xlsx
@@ -410,19 +410,19 @@
     <t>YRKDK7PA5G</t>
   </si>
   <si>
-    <t>Veltlínské zelené - Lampelberg 2024 VOC</t>
+    <t>Veltlínské zelené - Volné pole 2025 VOC</t>
   </si>
   <si>
     <t xml:space="preserve">Vinařství LAHOFER, a.s. </t>
   </si>
   <si>
-    <t>LAH.0525</t>
-  </si>
-  <si>
-    <t>Víno zlatavě-zelenkavé barvy, jehož vůni vévodí kořenitost a stopy bílého pepře doplněné o jemný mandlově-minerální nádech. V plné chuti vystupují do popředí především pepřnaté tóny protknuté lehkou kořenitostí a svěžím odstínem letního jablíčka.</t>
-  </si>
-  <si>
-    <t>YR678HX1OD</t>
+    <t>LAH.0566</t>
+  </si>
+  <si>
+    <t>Víno zlatavě-zelenkavé barvy, jehož vůni vévodí šťavnatost letního jablíčka se stopami bílého pepře doplněná o jemný mandlový nádech. V plné chuti vystupují do popředí především pikantní pepřnaté tóny. Dlouhý příjemně minerální závěr.</t>
+  </si>
+  <si>
+    <t>YRKY8039JJ</t>
   </si>
   <si>
     <t>VINAŘSTVÍ DOBROVOLNÝ</t>
@@ -3038,7 +3038,7 @@
         <v>24</v>
       </c>
       <c r="E16" t="n">
-        <v>2024.0</v>
+        <v>2025.0</v>
       </c>
       <c r="F16" t="s">
         <v>47</v>
@@ -3068,13 +3068,13 @@
         <v>134</v>
       </c>
       <c r="O16" t="n">
-        <v>13.0</v>
+        <v>12.0</v>
       </c>
       <c r="P16" t="n">
-        <v>4.1</v>
+        <v>3.7</v>
       </c>
       <c r="Q16" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="R16" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
Aktualizovat data vinné karty z ERP (2026-10-27)
</commit_message>
<xml_diff>
--- a/data/Enoteka_pozice.xlsx
+++ b/data/Enoteka_pozice.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1706" uniqueCount="647">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1704" uniqueCount="648">
   <si>
     <t>Je_v_ENO</t>
   </si>
@@ -1869,94 +1869,97 @@
     <t>YRU9YO3RVF</t>
   </si>
   <si>
-    <t>VIH.0256</t>
-  </si>
-  <si>
-    <t>49,5</t>
-  </si>
-  <si>
-    <t>YRXBX4DRUN</t>
-  </si>
-  <si>
-    <t>ZNO.0472</t>
-  </si>
-  <si>
-    <t>14,4</t>
-  </si>
-  <si>
-    <t>Je krásný, typický, odrůdový, zaujme hned na první přivonění. Najdete v něm květ bezu, zralý angrešt nebo černý rybíz. Chuť je bohatá, čistá a harmonická, s tóny manga, liči nebo kompotovaného ananasu. Milovníky Hibernalu toto víno jistě potěší.</t>
-  </si>
-  <si>
-    <t>YRXK2JW722</t>
-  </si>
-  <si>
-    <t>Cuvée Šaldec</t>
-  </si>
-  <si>
-    <t>PAJ.0160</t>
-  </si>
-  <si>
-    <t>Příjemné nekomplikované víno respektující terroir a atmosféru Nového Šaldorfa. Víno s nižším obsahem alkoholu a příjemným zbytkovým cukrem na horní hranici polosuchého vína. Postavené na místních odrůdách tak, aby bylo hravé, příjemné a odpočinkové. Osloví především vychutnávače polosuchých vín.</t>
-  </si>
-  <si>
-    <t>YRKU4320HT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sauvignon gris </t>
-  </si>
-  <si>
-    <t>HAN.0197</t>
-  </si>
-  <si>
-    <t>Sauvignon gris</t>
-  </si>
-  <si>
-    <t>Sauvignon gris - Volné pole - 2020 p.s.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sauvignon Gris neboli Sauvignon šedý je odrůdová mutace Sauvignonu Blanc, s nímž má podobný charakterový projev. Tento Sauvignon šedý je navíc vínem panenským - již dvouletá výsadba nám v roce 2020 dala první úrodu! Osloví vás barvou lipového květu, upoutá vůní josty, bělomasé broskve a jemným citrusovým aromatem. V ústech ucítíte příjemnou živost, svěží a vyváženou chuť angreštu a citrusových plodů podtrhuje křupavá kyselinka, která potěší milovníky opravdu suchých vín.  </t>
-  </si>
-  <si>
-    <t>YR5D0ALZL9</t>
-  </si>
-  <si>
-    <t>Rinot</t>
-  </si>
-  <si>
-    <t>PLA.0141</t>
-  </si>
-  <si>
-    <t>2,1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Suché bílé víno odrůdy Rinot ročníku 2024, pozdní sběr, z vinařství Jana Plačka z Moravských Bránic. Barva vína je živě žlutozlatá. Decentní vůně se  postupně uvolňuje a cítíme čerstvě upečený chléb, zahradní ovoce a ryngle. Chuť koresponduje s vůní, je jemná, decentní, se sladěným zbytkovým cukrem a kyselinkou. </t>
-  </si>
-  <si>
-    <t>YRBIPP0OBZ</t>
-  </si>
-  <si>
-    <t>PINK</t>
-  </si>
-  <si>
-    <t>ART.0085</t>
-  </si>
-  <si>
-    <t>Pink 2022 je jemně ovocný s nádechem po lesních plodech a třešních přecházejícím do decentní, jemné kořenitosti. Na jazyce svěží a ovocný s překvapivě plným tělem.</t>
-  </si>
-  <si>
-    <t>YR9T6K5XSY</t>
-  </si>
-  <si>
-    <t>Rulandské modré - Volné pole 2021 v.h.</t>
-  </si>
-  <si>
-    <t>WAL.0395</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Víno tmavé cihlově červené barvy, s vůní sladké mleté papriky a sušeného tabákového listu. Vysoce extraktivní chuť odkazuje na vyzrálost hroznů a částečné ležení v dubovém sudu. Je robustní, jemně kořenitá, s dlouhou perzistencí a lehce nasládlou vanilkovou stopou v jejím závěru. Víno má velmi dobré předpoklady k další archivaci a nazrávání na lahvi. </t>
-  </si>
-  <si>
-    <t>YRZMJLNXEN</t>
+    <t>Rizvanec</t>
+  </si>
+  <si>
+    <t>PAJ.0167</t>
+  </si>
+  <si>
+    <t>Krásný mladý Rizvaneček (kříženec ryzlinku a sylvánu), šťavnatý, svěží s lehkým dotekem zbytkového cukru do chladných podzimních večerů.</t>
+  </si>
+  <si>
+    <t>YRA8QA5OOD</t>
+  </si>
+  <si>
+    <t>První letošní Svatovavřinecké rosé</t>
+  </si>
+  <si>
+    <t>ZNO.0517</t>
+  </si>
+  <si>
+    <t>12,1</t>
+  </si>
+  <si>
+    <t>Svatovavřinecké</t>
+  </si>
+  <si>
+    <t>Svěží mladé víno odrůdy Svatovavřinecké lehkého typu v polosuché variantě ze Znovínu Znojmo.</t>
+  </si>
+  <si>
+    <t>YRD3CPXHTJ</t>
+  </si>
+  <si>
+    <t>První letošní Sauvignon 2026</t>
+  </si>
+  <si>
+    <t>ZNO.0518</t>
+  </si>
+  <si>
+    <t>Aromatické mladé víno odrůdy Sauvignon v suché variantě ze Znovínu Znojmo.</t>
+  </si>
+  <si>
+    <t>YR34RPYDFB</t>
+  </si>
+  <si>
+    <t>Martin Růžový 2026 m.z.v.</t>
+  </si>
+  <si>
+    <t>HAN.0286</t>
+  </si>
+  <si>
+    <t>Modrý Portugal</t>
+  </si>
+  <si>
+    <t>Polosuché rosé odrůdy Modrý Portugal. Vůni vévodí pivoňky a třešně srdcovky. Ty hrají prim i v jeho lahodné chuti podpořené mladistvou, svěží kyselinkou.</t>
+  </si>
+  <si>
+    <t>YR08A0K8RB</t>
+  </si>
+  <si>
+    <t>Martin Bílý 2026 m.z.v.</t>
+  </si>
+  <si>
+    <t>HAN.0285</t>
+  </si>
+  <si>
+    <t>Atraktivní polosladký Hibernal se svěží vůní citrusů a s neskutečně šťavnatou a ovocitou chutí připomínající žlutomasou broskev nebo pomelo.</t>
+  </si>
+  <si>
+    <t>YRX1CI1J30</t>
+  </si>
+  <si>
+    <t>LAHOFERka 26 m.z.v.</t>
+  </si>
+  <si>
+    <t>LAH.0601</t>
+  </si>
+  <si>
+    <t>Růžové víno z odrůdy Svatovavřinecké okouzlí jemnou vůní jahod se smetanou s elegantní stopou růží. V chuti se přidávají šťavnaté tóny lesních jahod a malin provázené svěží kyselinkou.</t>
+  </si>
+  <si>
+    <t>YRGDMUWR45</t>
+  </si>
+  <si>
+    <t>LAHOFER 26 m.z.v.</t>
+  </si>
+  <si>
+    <t>LAH.0600</t>
+  </si>
+  <si>
+    <t>Svěží bílé cuvée z odrůd Müller Thurgau a Muškát moravský s atraktivním muškátově-vanilkovým aroma. V chuti tóny mandarinky a černého rybízu podpořené příjemně živelnou kyselinkou.</t>
+  </si>
+  <si>
+    <t>YROGZFT21L</t>
   </si>
 </sst>
 </file>
@@ -9764,64 +9767,64 @@
         <v>114.0</v>
       </c>
       <c r="C115" t="s">
-        <v>218</v>
+        <v>617</v>
       </c>
       <c r="D115" t="s">
-        <v>329</v>
+        <v>220</v>
       </c>
       <c r="E115" t="n">
-        <v>2025.0</v>
+        <v>2026.0</v>
       </c>
       <c r="F115" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G115" t="s">
-        <v>48</v>
+        <v>148</v>
       </c>
       <c r="H115" t="s">
-        <v>27</v>
+        <v>152</v>
       </c>
       <c r="I115" t="n">
-        <v>16.0</v>
+        <v>0.0</v>
       </c>
       <c r="J115" t="n">
-        <v>36.0</v>
+        <v>0.0</v>
       </c>
       <c r="K115" t="n">
-        <v>57.0</v>
+        <v>0.0</v>
       </c>
       <c r="L115" t="n">
         <v>70.0</v>
       </c>
       <c r="M115" t="n">
-        <v>199.0</v>
+        <v>175.0</v>
       </c>
       <c r="N115" t="s">
+        <v>618</v>
+      </c>
+      <c r="O115" t="s">
+        <v>242</v>
+      </c>
+      <c r="P115" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q115" t="s">
+        <v>99</v>
+      </c>
+      <c r="R115" t="s">
+        <v>32</v>
+      </c>
+      <c r="S115" t="s">
+        <v>33</v>
+      </c>
+      <c r="T115" t="s">
         <v>617</v>
       </c>
-      <c r="O115" t="s">
-        <v>40</v>
-      </c>
-      <c r="P115" t="s">
-        <v>618</v>
-      </c>
-      <c r="Q115" t="s">
-        <v>42</v>
-      </c>
-      <c r="R115" t="s">
-        <v>32</v>
-      </c>
-      <c r="S115" t="s">
-        <v>218</v>
-      </c>
-      <c r="T115" t="s">
-        <v>218</v>
-      </c>
       <c r="U115" t="s">
-        <v>152</v>
+        <v>619</v>
       </c>
       <c r="V115" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
     </row>
     <row r="116">
@@ -9832,64 +9835,64 @@
         <v>115.0</v>
       </c>
       <c r="C116" t="s">
-        <v>75</v>
+        <v>621</v>
       </c>
       <c r="D116" t="s">
         <v>220</v>
       </c>
       <c r="E116" t="n">
-        <v>2025.0</v>
+        <v>2026.0</v>
       </c>
       <c r="F116" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G116" t="s">
-        <v>96</v>
+        <v>562</v>
       </c>
       <c r="H116" t="s">
         <v>27</v>
       </c>
       <c r="I116" t="n">
-        <v>16.0</v>
+        <v>12.0</v>
       </c>
       <c r="J116" t="n">
-        <v>36.0</v>
+        <v>24.0</v>
       </c>
       <c r="K116" t="n">
-        <v>57.0</v>
+        <v>41.0</v>
       </c>
       <c r="L116" t="n">
         <v>70.0</v>
       </c>
       <c r="M116" t="n">
-        <v>180.0</v>
+        <v>99.0</v>
       </c>
       <c r="N116" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="O116" t="s">
-        <v>78</v>
+        <v>265</v>
       </c>
       <c r="P116" t="s">
+        <v>623</v>
+      </c>
+      <c r="Q116" t="s">
+        <v>232</v>
+      </c>
+      <c r="R116" t="s">
+        <v>374</v>
+      </c>
+      <c r="S116" t="s">
+        <v>624</v>
+      </c>
+      <c r="T116" t="s">
         <v>621</v>
       </c>
-      <c r="Q116" t="s">
-        <v>99</v>
-      </c>
-      <c r="R116" t="s">
-        <v>32</v>
-      </c>
-      <c r="S116" t="s">
-        <v>75</v>
-      </c>
-      <c r="T116" t="s">
-        <v>75</v>
-      </c>
       <c r="U116" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="V116" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
     </row>
     <row r="117">
@@ -9900,64 +9903,64 @@
         <v>116.0</v>
       </c>
       <c r="C117" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="D117" t="s">
-        <v>220</v>
+        <v>24</v>
       </c>
       <c r="E117" t="n">
-        <v>2023.0</v>
+        <v>2026.0</v>
       </c>
       <c r="F117" t="s">
         <v>25</v>
       </c>
       <c r="G117" t="s">
-        <v>148</v>
+        <v>562</v>
       </c>
       <c r="H117" t="s">
-        <v>152</v>
+        <v>27</v>
       </c>
       <c r="I117" t="n">
-        <v>0.0</v>
+        <v>12.0</v>
       </c>
       <c r="J117" t="n">
-        <v>0.0</v>
+        <v>24.0</v>
       </c>
       <c r="K117" t="n">
-        <v>0.0</v>
+        <v>41.0</v>
       </c>
       <c r="L117" t="n">
         <v>70.0</v>
       </c>
       <c r="M117" t="n">
-        <v>180.0</v>
+        <v>99.0</v>
       </c>
       <c r="N117" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
       <c r="O117" t="s">
         <v>40</v>
       </c>
-      <c r="P117" t="n">
-        <v>16.0</v>
+      <c r="P117" t="s">
+        <v>422</v>
       </c>
       <c r="Q117" t="s">
-        <v>31</v>
+        <v>156</v>
       </c>
       <c r="R117" t="s">
         <v>32</v>
       </c>
       <c r="S117" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="T117" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="U117" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="V117" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
     </row>
     <row r="118">
@@ -9968,16 +9971,16 @@
         <v>117.0</v>
       </c>
       <c r="C118" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="D118" t="s">
-        <v>24</v>
+        <v>220</v>
       </c>
       <c r="E118" t="n">
-        <v>2020.0</v>
+        <v>2026.0</v>
       </c>
       <c r="F118" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="G118" t="s">
         <v>199</v>
@@ -9998,34 +10001,34 @@
         <v>70.0</v>
       </c>
       <c r="M118" t="n">
-        <v>150.0</v>
+        <v>140.0</v>
       </c>
       <c r="N118" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="O118" t="n">
-        <v>12.0</v>
+        <v>11.0</v>
       </c>
       <c r="P118" t="n">
-        <v>0.7</v>
+        <v>11.2</v>
       </c>
       <c r="Q118" t="n">
-        <v>6.9</v>
+        <v>5.7</v>
       </c>
       <c r="R118" t="s">
-        <v>32</v>
+        <v>374</v>
       </c>
       <c r="S118" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="T118" t="s">
         <v>631</v>
       </c>
       <c r="U118" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="V118" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
     </row>
     <row r="119">
@@ -10036,64 +10039,64 @@
         <v>118.0</v>
       </c>
       <c r="C119" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="D119" t="s">
-        <v>24</v>
+        <v>283</v>
       </c>
       <c r="E119" t="n">
-        <v>2024.0</v>
+        <v>2026.0</v>
       </c>
       <c r="F119" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="G119" t="s">
-        <v>154</v>
+        <v>199</v>
       </c>
       <c r="H119" t="s">
         <v>27</v>
       </c>
       <c r="I119" t="n">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
       <c r="J119" t="n">
-        <v>36.0</v>
+        <v>30.0</v>
       </c>
       <c r="K119" t="n">
-        <v>57.0</v>
+        <v>49.0</v>
       </c>
       <c r="L119" t="n">
         <v>70.0</v>
       </c>
       <c r="M119" t="n">
-        <v>182.0</v>
+        <v>130.0</v>
       </c>
       <c r="N119" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="O119" t="n">
-        <v>13.0</v>
-      </c>
-      <c r="P119" t="s">
+        <v>10.0</v>
+      </c>
+      <c r="P119" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="Q119" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R119" t="s">
+        <v>32</v>
+      </c>
+      <c r="S119" t="s">
+        <v>75</v>
+      </c>
+      <c r="T119" t="s">
         <v>636</v>
       </c>
-      <c r="Q119" t="s">
-        <v>114</v>
-      </c>
-      <c r="R119" t="s">
-        <v>32</v>
-      </c>
-      <c r="S119" t="s">
-        <v>634</v>
-      </c>
-      <c r="T119" t="s">
-        <v>634</v>
-      </c>
       <c r="U119" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="V119" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
     </row>
     <row r="120">
@@ -10104,19 +10107,19 @@
         <v>119.0</v>
       </c>
       <c r="C120" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="D120" t="s">
-        <v>24</v>
+        <v>283</v>
       </c>
       <c r="E120" t="n">
-        <v>2022.0</v>
+        <v>2026.0</v>
       </c>
       <c r="F120" t="s">
         <v>25</v>
       </c>
       <c r="G120" t="s">
-        <v>580</v>
+        <v>133</v>
       </c>
       <c r="H120" t="s">
         <v>27</v>
@@ -10134,34 +10137,34 @@
         <v>70.0</v>
       </c>
       <c r="M120" t="n">
-        <v>175.0</v>
+        <v>140.0</v>
       </c>
       <c r="N120" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="O120" t="n">
-        <v>12.0</v>
+        <v>10.0</v>
       </c>
       <c r="P120" t="n">
-        <v>3.0</v>
-      </c>
-      <c r="Q120" t="s">
-        <v>173</v>
+        <v>31.5</v>
+      </c>
+      <c r="Q120" t="n">
+        <v>6.4</v>
       </c>
       <c r="R120" t="s">
         <v>374</v>
       </c>
       <c r="S120" t="s">
-        <v>397</v>
+        <v>624</v>
       </c>
       <c r="T120" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="U120" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="V120" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
     </row>
     <row r="121">
@@ -10172,19 +10175,19 @@
         <v>120.0</v>
       </c>
       <c r="C121" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="D121" t="s">
-        <v>24</v>
+        <v>220</v>
       </c>
       <c r="E121" t="n">
-        <v>2021.0</v>
+        <v>2026.0</v>
       </c>
       <c r="F121" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G121" t="s">
-        <v>56</v>
+        <v>133</v>
       </c>
       <c r="H121" t="s">
         <v>27</v>
@@ -10202,34 +10205,34 @@
         <v>70.0</v>
       </c>
       <c r="M121" t="n">
-        <v>160.0</v>
+        <v>130.0</v>
       </c>
       <c r="N121" t="s">
+        <v>645</v>
+      </c>
+      <c r="O121" t="n">
+        <v>11.0</v>
+      </c>
+      <c r="P121" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="Q121" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="R121" t="s">
+        <v>32</v>
+      </c>
+      <c r="S121" t="s">
+        <v>191</v>
+      </c>
+      <c r="T121" t="s">
         <v>644</v>
       </c>
-      <c r="O121" t="n">
-        <v>14.0</v>
-      </c>
-      <c r="P121" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="Q121" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="R121" t="s">
-        <v>405</v>
-      </c>
-      <c r="S121" t="s">
-        <v>406</v>
-      </c>
-      <c r="T121" t="s">
-        <v>643</v>
-      </c>
       <c r="U121" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="V121" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aktualizovat data vinné karty z ERP (2026-10-30)
</commit_message>
<xml_diff>
--- a/data/Enoteka_pozice.xlsx
+++ b/data/Enoteka_pozice.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1704" uniqueCount="648">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1701" uniqueCount="659">
   <si>
     <t>Je_v_ENO</t>
   </si>
@@ -1311,25 +1311,34 @@
     <t>YRI3M8SQWI</t>
   </si>
   <si>
-    <t>VAN.0148</t>
-  </si>
-  <si>
-    <t>Suché bílé víno odrůdy Veltlínské zelené, 2025, VOC z vinařství Vaněk. Pepřnaté víno s výraznou kořenitostí, mandlovými tóny a vyšší svěží kyselinkou, která mu dodává šťavnatost. Charakteristická je pro něj mineralita, tóny žlutého melounu či akátového medu.</t>
-  </si>
-  <si>
-    <t>YRXEDZJMGX</t>
-  </si>
-  <si>
-    <t>ZNO.0478</t>
-  </si>
-  <si>
-    <t>0,6</t>
-  </si>
-  <si>
-    <t>Ve vůni dominuje bílý pepř a květinové tóny, které připomínají rozkvetlou jarní louku. V ústech vás potěší svěžest a výrazný ovocný projev. Hledejte broskve, zelené jablka nebo máslové hrušky.</t>
-  </si>
-  <si>
-    <t>YRCZ6MVAR2</t>
+    <t>TAO.0202</t>
+  </si>
+  <si>
+    <t>Frankovka Na nivách</t>
+  </si>
+  <si>
+    <t>Červené suché víno odrůdy Frankovka ročníku 2023 z Dolních Kounice z Oulehla vinařství. Frankovka je pro tuto oblast vlakovou lodí, je elegantní, plná a aromatická.</t>
+  </si>
+  <si>
+    <t>YR21P871KA</t>
+  </si>
+  <si>
+    <t>Rulandské modré Barrel</t>
+  </si>
+  <si>
+    <t>NES.0012</t>
+  </si>
+  <si>
+    <t>14,0</t>
+  </si>
+  <si>
+    <t>4,7</t>
+  </si>
+  <si>
+    <t>Bohaté komplexní víno odrůdy Rulandské modré, Special Barrel, ročníku 2024 z Vinařství Nešetřil ze Znojma. Kvalitní hrozny, šetrné zacházení a zrání na sudu dávají vínu plnost a harmoničnost, je tedy je právem kandidátem do Salonu vín 2027. Vino zrálo 20 měsíců v barikových sudech.</t>
+  </si>
+  <si>
+    <t>YRNPY0CP8P</t>
   </si>
   <si>
     <t>SPA.0198</t>
@@ -1344,130 +1353,158 @@
     <t>YRKMQCFA15</t>
   </si>
   <si>
-    <t>PAJ.0162</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typický veltlínek ze Znojemska, svěží květinovo - ovocný profil s harmonickou kyselinkou a krásnou stopou bílého pepře. Ideální jemný společník k předkrmu, navození vinné atmosféry či relaxaci. </t>
-  </si>
-  <si>
-    <t>YRV86DFXSW</t>
-  </si>
-  <si>
-    <t>HOD.0089</t>
+    <t>Veltlínské zelené - Pozdravy z NP Podyjí</t>
+  </si>
+  <si>
+    <t>KOR.0223</t>
+  </si>
+  <si>
+    <t>6,3</t>
+  </si>
+  <si>
+    <t>Barva je sytá, zlatavá. Velmi dobrá viskozita. V aromatice můžeme najít komplexní veltlínské zelené se znaky citrusů, žlutého ovoce a bílého pepře. Chuť je středně plná převážně se znaky vyzrálého zahradního ovoce. Delší perzistence.</t>
+  </si>
+  <si>
+    <t>YRIC6Z1HE2</t>
+  </si>
+  <si>
+    <t>Pinot Blanc 2024</t>
+  </si>
+  <si>
+    <t>KOR.0228</t>
+  </si>
+  <si>
+    <t>3,4</t>
+  </si>
+  <si>
+    <t>Pinot Blanc</t>
+  </si>
+  <si>
+    <t>Víno kvasilo a zrálo v sudech o objemu 400L. Vrstevnaté a komplexní víno s charakterem. Má zlatožlutou barvu. Aromatika je široká s tóny pečené kůrky chleba a zralého žlutého ovoce. Můžeme zde najít i lehkou stopu medové plástve. Chuť je harmonická a minerální s lehkou stopou zrání v dřevěných sudech.</t>
+  </si>
+  <si>
+    <t>YRZOBGFYDB</t>
+  </si>
+  <si>
+    <t>Ryzlink rýnský - U Hájku 2025 VOC</t>
+  </si>
+  <si>
+    <t>LAH.0582</t>
+  </si>
+  <si>
+    <t>Elegantní ryzlink světle zlaté barvy, jehož vůni dominují tóny sušených meruněk. Výrazná ovocná chuť šťavnatých rynglí dokonale harmonizuje s pikantní kyselinkou a delikátním minerálním závěrem. Zráním na lahvi budou v tomto ryzlinku sílit petrolejové tóny.</t>
+  </si>
+  <si>
+    <t>YRC8UPYB9W</t>
+  </si>
+  <si>
+    <t>Rulandské bílé - Volné pole 2024 p.s.</t>
+  </si>
+  <si>
+    <t>HAN.0275</t>
+  </si>
+  <si>
+    <t>Víno jiskrné perleťové barvy, v jehož vůni se kromě převládající stopy čerstvého másla otiskuje i tříměsíční ležení v dubovém sudu, které mu dodalo jemně nasládlý vanilkový tón. V ústech je elegantní, vytříbenou chuť definují jemná ovocitost a mineralita.</t>
+  </si>
+  <si>
+    <t>YRWSWPTXB8</t>
+  </si>
+  <si>
+    <t>Hibernal privileg</t>
+  </si>
+  <si>
+    <t>PLA.0157</t>
+  </si>
+  <si>
+    <t>Víno s jásavou žluto zelenkavou barvou. Osloví vás svou výraznou intenzivní vůní citrusů, angreštu, černého rybízu, bylin, a to výrazný projev jarní kopřivy nebo lipového květu. Chuť vína je lehká, šťavnatá, svěží, s jemnou kyselinkou a nepatrným zbytkovým cukrem.</t>
+  </si>
+  <si>
+    <t>YRIPDM8FUB</t>
+  </si>
+  <si>
+    <t>SPA.0203</t>
+  </si>
+  <si>
+    <t>Z hroznů sklizených koncem října, kdy dosáhly optimální zralosti. Po pomletí a lisování i se stopkami probíhalo kvašení s použitím čisté kultury kvasinek. Víno kvasilo a zrálo výhradně v nerezových tancích, aby si zachovalo svěžest a čistotu odrůdového projevu.
+Ve vůni se objevují tóny zralých meruněk s jemným petrolejovým nádechem. Chuť je plná, ovocná a minerální, s vyváženou kyselinou a příjemným zbytkovým cukrem, který vytváří harmonický a svěží dojem v závěru.</t>
+  </si>
+  <si>
+    <t>YRUI5T7O5H</t>
+  </si>
+  <si>
+    <t>VIH.0260</t>
+  </si>
+  <si>
+    <t>Suché bílé víno odrůdy Sauvignon, 2025, VOC z vinařství VINICE-HNANICE.  Aromatické víno s výrazným projevem angreštu, rybízu, broskví a černého bezu. Víno se vyznačuje vysokou kvalitou, mineralitou a typickým terroirem, často s ovocným profilem a svěží kyselinkou.</t>
+  </si>
+  <si>
+    <t>YRVHZM4KO8</t>
+  </si>
+  <si>
+    <t>PAJ.0163</t>
   </si>
   <si>
     <t>7,4</t>
   </si>
   <si>
-    <t>Suché bílé víno odrůdy Veltlínské zelené, 2025, VOC z vinařství Zemědělské družstvo Hodonice - Tasovické vinařství. Pepřnaté víno s výraznou kořenitostí, mandlovými tóny a vyšší svěží kyselinkou, která mu dodává šťavnatost. Charakteristická je pro něj mineralita, tóny žlutého melounu či akátového medu.</t>
-  </si>
-  <si>
-    <t>YRZ1JVK4VS</t>
-  </si>
-  <si>
-    <t>HAL.0021</t>
-  </si>
-  <si>
-    <t>suché bílé víno odrůdy Sauvignon, 2025, VOC z vinařství HALKOCI. Aromatické víno s výrazným projevem angreštu, rybízu, broskví a černého bezu. Víno se vyznačuje vysokou kvalitou, mineralitou a typickým terroirem, často s ovocným profilem a svěží kyselinkou.</t>
-  </si>
-  <si>
-    <t>YRGU9HQU99</t>
-  </si>
-  <si>
-    <t>SIM.0088</t>
-  </si>
-  <si>
-    <t>1,7</t>
-  </si>
-  <si>
-    <t>suché bílé víno odrůdy Sauvignon, 2025, VOC z vinařství SIMENON. Suché aromatické víno ze znojemského regionu s výrazným projevem angreštu, rybízu, broskví a černého bezu. Víno se vyznačuje vysokou kvalitou, mineralitou a typickým terroirem, často s ovocným profilem a svěží kyselinkou.</t>
-  </si>
-  <si>
-    <t>YRATC09R45</t>
-  </si>
-  <si>
-    <t>VIH.0260</t>
-  </si>
-  <si>
-    <t>Suché bílé víno odrůdy Sauvignon, 2025, VOC z vinařství VINICE-HNANICE.  Aromatické víno s výrazným projevem angreštu, rybízu, broskví a černého bezu. Víno se vyznačuje vysokou kvalitou, mineralitou a typickým terroirem, často s ovocným profilem a svěží kyselinkou.</t>
-  </si>
-  <si>
-    <t>YRVHZM4KO8</t>
-  </si>
-  <si>
-    <t>SPA.0199</t>
-  </si>
-  <si>
-    <t>Suché bílé víno odrůda Sauvignon, 2025, VOC z Vinařství rodiny Špalkovy. Aromatické víno znojemského regionu s výrazným projevem angreštu, rybízu, broskví a černého bezu. Víno se vyznačuje vysokou kvalitou, mineralitou a typickým terroirem, často s ovocným profilem a svěží kyselinkou.</t>
-  </si>
-  <si>
-    <t>YR6LSMCSJ8</t>
-  </si>
-  <si>
-    <t>PAJ.0163</t>
-  </si>
-  <si>
     <t>Suché bílé víno odrůdy Sauvignon, 2025, VOC z vinařství Pijálek&amp;Jäger. Aromatické víno s výrazným projevem angreštu, rybízu, broskví a černého bezu. Víno se vyznačuje vysokou kvalitou, mineralitou a typickým terroirem, často s ovocným profilem a svěží kyselinkou.</t>
   </si>
   <si>
     <t>YRK2VWNMSE</t>
   </si>
   <si>
-    <t>SIM.0086</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ryzlink rýnský VOC </t>
-  </si>
-  <si>
-    <t>Suché bílé víno odrůdy Ryzlink rýnský ročníku 2025, VOC Znojmo, z vinařství SIMENON. Suché, minerální a svěží víno s výraznou ovocnou aromatikou (meruňky, citrusy, kdoule) a pikantní kyselinkou. Vyznačuje se lipovými tóny, kořenitostí a často jemným petrolejovým nádechem v dochuti.</t>
-  </si>
-  <si>
-    <t>YRDSGIGCNV</t>
-  </si>
-  <si>
-    <t>VAN.0151</t>
-  </si>
-  <si>
-    <t>3,6</t>
-  </si>
-  <si>
-    <t>suché bílé víno odrůdy Ryzlink rýnský, 2025, VOC z vinařství Vaněk. Minerální a svěží víno s výraznou ovocnou aromatikou (meruňky, citrusy, kdoule) a pikantní kyselinkou. Vyznačuje se lipovými tóny, kořenitostí a často jemným petrolejovým nádechem v dochuti.</t>
-  </si>
-  <si>
-    <t>YRLCX0IRW5</t>
-  </si>
-  <si>
-    <t>ZNO.0480</t>
-  </si>
-  <si>
-    <t>Suché bílé víno odrůdy Ryzlink rýnský, 2025, VOC z vinařství ZNOVÍN ZNOJMO. Minerální a svěží víno s výraznou ovocnou aromatikou (meruňky, citrusy, kdoule) a pikantní kyselinkou. Vyznačuje se lipovými tóny, kořenitostí a často jemným petrolejovým nádechem v dochuti.</t>
-  </si>
-  <si>
-    <t>YRLHISRK7W</t>
-  </si>
-  <si>
-    <t>VSL.0145</t>
-  </si>
-  <si>
-    <t>11,7</t>
-  </si>
-  <si>
-    <t>suché bílé víno odrůdy Ryzlink rýnský, 2025, VOC z vinařství Vinné sklepy Lechovice. Minerální a svěží víno s výraznou ovocnou aromatikou (meruňky, citrusy, kdoule) a pikantní kyselinkou. Vyznačuje se lipovými tóny, kořenitostí a často jemným petrolejovým nádechem v dochuti.</t>
-  </si>
-  <si>
-    <t>YRCQIPM6VQ</t>
-  </si>
-  <si>
-    <t>AMP.0185</t>
-  </si>
-  <si>
-    <t>10,1</t>
-  </si>
-  <si>
-    <t>Polosuché bílé víno odrůdy Ryzlink rýnský, 2025, VOC z vinařství AMPELOS. Minerální a svěží víno s výraznými lipovými tóny a pikantní kyselinkou, v dochutí s lehce petrolejovými tóny.</t>
-  </si>
-  <si>
-    <t>YRQI0NUJTE</t>
+    <t>Ryzlink rýnský - U Hájku 2024 VOC</t>
+  </si>
+  <si>
+    <t>LAH.0543</t>
+  </si>
+  <si>
+    <t>Elegantní ryzlink zlatavé barvy, jehož chuti i vůni dominují tóny čerstvých meruněk. Výraznou ovocnou šťavnatost skvěle doplňuje zbytkový cukr v dokonalé harmonii s pikantní kyselinkou a delším minerálním závěrem. Zráním na lahvi budou v tomto ryzlinku sílit petrolejové tóny.</t>
+  </si>
+  <si>
+    <t>YR6PJY8U34</t>
+  </si>
+  <si>
+    <t>ZNOVÍN ZNOJMO a.s. - NEPOUŽÍVAT</t>
+  </si>
+  <si>
+    <t>ZNO.0444</t>
+  </si>
+  <si>
+    <t>27,1</t>
+  </si>
+  <si>
+    <t>Hned po přivonění ucítíte med, máslové sušenky, rozinky a kořenitost. V ústech je nádherně plné, harmonické a opojné, s tóny kandovaného ovoce, sladkého koření, vanilky nebo kompotovaných rynglí. Víno má neobyčejně dlouhou dochuť.</t>
+  </si>
+  <si>
+    <t>YRKLTR8KP6</t>
+  </si>
+  <si>
+    <t>PAJ.0165</t>
+  </si>
+  <si>
+    <t>32,1</t>
+  </si>
+  <si>
+    <t>Typický, aromatický a extraktivní tramín, plný květů a koření v kombinaci s velkým zbytkovým cukrem, zakončený velmi příjemnou kyselinkou.</t>
+  </si>
+  <si>
+    <t>YRQNB6NYSQ</t>
+  </si>
+  <si>
+    <t>ZNO.0456</t>
+  </si>
+  <si>
+    <t>80,9</t>
+  </si>
+  <si>
+    <t>7,8</t>
+  </si>
+  <si>
+    <t>Víno je nádherně ušlechtilé, plné, mohutné a neodolatelné. Uchvátí zlatavou barvou i dokonalým souzněním svůdného zbytkového cukru a svěžích kyselin. Ve vůni i chuti hledejte med, rozinky, vanilku, sladké koření a kandované ovoce.</t>
+  </si>
+  <si>
+    <t>YR4SUL03PN</t>
   </si>
   <si>
     <t>Ryzlink vlašský - WAVE Beton</t>
@@ -1489,6 +1526,9 @@
     <t>HOR.0155</t>
   </si>
   <si>
+    <t>0,6</t>
+  </si>
+  <si>
     <t xml:space="preserve">bílé suché víno, směs odrůd Veltlínské zelené a Ryzlink rýnský, ročník 2024 z vinařství Víno Hort. Kořenité minerální víno, zrání ve granitovém vejci. </t>
   </si>
   <si>
@@ -1517,9 +1557,6 @@
   </si>
   <si>
     <t>DNT.0004</t>
-  </si>
-  <si>
-    <t>6,3</t>
   </si>
   <si>
     <t xml:space="preserve">naturální oranžové suché víno odrůdy Pálava. Víno je ze sklizně ročníků 2023 a 2024, je vyráběno přírodní metodou s velmi nízkým obsahem oxidu siřičitého. </t>
@@ -1701,9 +1738,6 @@
   </si>
   <si>
     <t>Kerner - Pírko</t>
-  </si>
-  <si>
-    <t>ZNOVÍN ZNOJMO a.s. - NEPOUŽÍVAT</t>
   </si>
   <si>
     <t>ZNO.0453</t>
@@ -6843,19 +6877,19 @@
         <v>71.0</v>
       </c>
       <c r="C72" t="s">
-        <v>46</v>
+        <v>382</v>
       </c>
       <c r="D72" t="s">
         <v>24</v>
       </c>
       <c r="E72" t="n">
-        <v>2025.0</v>
+        <v>2023.0</v>
       </c>
       <c r="F72" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="G72" t="s">
-        <v>247</v>
+        <v>76</v>
       </c>
       <c r="H72" t="s">
         <v>27</v>
@@ -6873,34 +6907,34 @@
         <v>70.0</v>
       </c>
       <c r="M72" t="n">
-        <v>210.0</v>
+        <v>230.0</v>
       </c>
       <c r="N72" t="s">
         <v>432</v>
       </c>
       <c r="O72" t="s">
-        <v>90</v>
-      </c>
-      <c r="P72" t="n">
-        <v>3.0</v>
+        <v>112</v>
+      </c>
+      <c r="P72" t="s">
+        <v>411</v>
       </c>
       <c r="Q72" t="s">
-        <v>50</v>
+        <v>182</v>
       </c>
       <c r="R72" t="s">
-        <v>32</v>
+        <v>405</v>
       </c>
       <c r="S72" t="s">
-        <v>51</v>
+        <v>382</v>
       </c>
       <c r="T72" t="s">
-        <v>46</v>
+        <v>433</v>
       </c>
       <c r="U72" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="V72" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="73">
@@ -6911,64 +6945,64 @@
         <v>72.0</v>
       </c>
       <c r="C73" t="s">
-        <v>46</v>
+        <v>436</v>
       </c>
       <c r="D73" t="s">
         <v>24</v>
       </c>
       <c r="E73" t="n">
-        <v>2025.0</v>
+        <v>2024.0</v>
       </c>
       <c r="F73" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="G73" t="s">
-        <v>96</v>
+        <v>221</v>
       </c>
       <c r="H73" t="s">
-        <v>152</v>
+        <v>27</v>
       </c>
       <c r="I73" t="n">
-        <v>0.0</v>
+        <v>26.0</v>
       </c>
       <c r="J73" t="n">
-        <v>0.0</v>
+        <v>56.0</v>
       </c>
       <c r="K73" t="n">
-        <v>0.0</v>
+        <v>91.0</v>
       </c>
       <c r="L73" t="n">
         <v>70.0</v>
       </c>
       <c r="M73" t="n">
-        <v>190.0</v>
+        <v>490.0</v>
       </c>
       <c r="N73" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="O73" t="s">
-        <v>40</v>
+        <v>438</v>
       </c>
       <c r="P73" t="s">
+        <v>411</v>
+      </c>
+      <c r="Q73" t="s">
+        <v>439</v>
+      </c>
+      <c r="R73" t="s">
+        <v>405</v>
+      </c>
+      <c r="S73" t="s">
+        <v>406</v>
+      </c>
+      <c r="T73" t="s">
         <v>436</v>
       </c>
-      <c r="Q73" t="s">
-        <v>65</v>
-      </c>
-      <c r="R73" t="s">
-        <v>32</v>
-      </c>
-      <c r="S73" t="s">
-        <v>51</v>
-      </c>
-      <c r="T73" t="s">
-        <v>46</v>
-      </c>
       <c r="U73" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="V73" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="74">
@@ -7012,13 +7046,13 @@
         <v>240.0</v>
       </c>
       <c r="N74" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="O74" t="s">
         <v>40</v>
       </c>
       <c r="P74" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="Q74" t="s">
         <v>189</v>
@@ -7033,10 +7067,10 @@
         <v>46</v>
       </c>
       <c r="U74" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="V74" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
     </row>
     <row r="75">
@@ -7047,7 +7081,7 @@
         <v>74.0</v>
       </c>
       <c r="C75" t="s">
-        <v>46</v>
+        <v>446</v>
       </c>
       <c r="D75" t="s">
         <v>24</v>
@@ -7056,40 +7090,40 @@
         <v>2025.0</v>
       </c>
       <c r="F75" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="G75" t="s">
-        <v>148</v>
+        <v>402</v>
       </c>
       <c r="H75" t="s">
-        <v>152</v>
+        <v>27</v>
       </c>
       <c r="I75" t="n">
-        <v>0.0</v>
+        <v>16.0</v>
       </c>
       <c r="J75" t="n">
-        <v>0.0</v>
+        <v>36.0</v>
       </c>
       <c r="K75" t="n">
-        <v>0.0</v>
+        <v>57.0</v>
       </c>
       <c r="L75" t="n">
         <v>70.0</v>
       </c>
       <c r="M75" t="n">
-        <v>220.0</v>
+        <v>195.0</v>
       </c>
       <c r="N75" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="O75" t="s">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="P75" t="s">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="Q75" t="s">
-        <v>326</v>
+        <v>448</v>
       </c>
       <c r="R75" t="s">
         <v>32</v>
@@ -7098,13 +7132,13 @@
         <v>51</v>
       </c>
       <c r="T75" t="s">
-        <v>46</v>
+        <v>446</v>
       </c>
       <c r="U75" t="s">
-        <v>444</v>
+        <v>449</v>
       </c>
       <c r="V75" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
     </row>
     <row r="76">
@@ -7115,64 +7149,64 @@
         <v>75.0</v>
       </c>
       <c r="C76" t="s">
-        <v>46</v>
+        <v>451</v>
       </c>
       <c r="D76" t="s">
         <v>24</v>
       </c>
       <c r="E76" t="n">
-        <v>2025.0</v>
+        <v>2024.0</v>
       </c>
       <c r="F76" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="G76" t="s">
-        <v>194</v>
+        <v>402</v>
       </c>
       <c r="H76" t="s">
         <v>27</v>
       </c>
       <c r="I76" t="n">
-        <v>14.0</v>
+        <v>21.0</v>
       </c>
       <c r="J76" t="n">
-        <v>30.0</v>
+        <v>49.0</v>
       </c>
       <c r="K76" t="n">
-        <v>49.0</v>
+        <v>79.0</v>
       </c>
       <c r="L76" t="n">
         <v>70.0</v>
       </c>
       <c r="M76" t="n">
-        <v>170.0</v>
+        <v>345.0</v>
       </c>
       <c r="N76" t="s">
-        <v>446</v>
-      </c>
-      <c r="O76" t="n">
-        <v>11.0</v>
+        <v>452</v>
+      </c>
+      <c r="O76" t="s">
+        <v>112</v>
       </c>
       <c r="P76" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="Q76" t="s">
-        <v>71</v>
+        <v>114</v>
       </c>
       <c r="R76" t="s">
         <v>32</v>
       </c>
       <c r="S76" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="T76" t="s">
-        <v>46</v>
+        <v>454</v>
       </c>
       <c r="U76" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="V76" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
     </row>
     <row r="77">
@@ -7183,7 +7217,7 @@
         <v>76.0</v>
       </c>
       <c r="C77" t="s">
-        <v>193</v>
+        <v>457</v>
       </c>
       <c r="D77" t="s">
         <v>24</v>
@@ -7195,52 +7229,52 @@
         <v>47</v>
       </c>
       <c r="G77" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="H77" t="s">
-        <v>152</v>
+        <v>27</v>
       </c>
       <c r="I77" t="n">
-        <v>0.0</v>
+        <v>16.0</v>
       </c>
       <c r="J77" t="n">
-        <v>0.0</v>
+        <v>36.0</v>
       </c>
       <c r="K77" t="n">
-        <v>0.0</v>
+        <v>57.0</v>
       </c>
       <c r="L77" t="n">
         <v>70.0</v>
       </c>
       <c r="M77" t="n">
-        <v>249.0</v>
+        <v>205.0</v>
       </c>
       <c r="N77" t="s">
-        <v>450</v>
+        <v>458</v>
       </c>
       <c r="O77" t="n">
-        <v>12.0</v>
-      </c>
-      <c r="P77" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q77" t="s">
-        <v>99</v>
+        <v>12.5</v>
+      </c>
+      <c r="P77" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>7.0</v>
       </c>
       <c r="R77" t="s">
         <v>32</v>
       </c>
       <c r="S77" t="s">
-        <v>43</v>
+        <v>100</v>
       </c>
       <c r="T77" t="s">
-        <v>193</v>
+        <v>457</v>
       </c>
       <c r="U77" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
       <c r="V77" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
     </row>
     <row r="78">
@@ -7251,19 +7285,19 @@
         <v>77.0</v>
       </c>
       <c r="C78" t="s">
-        <v>193</v>
+        <v>461</v>
       </c>
       <c r="D78" t="s">
         <v>24</v>
       </c>
       <c r="E78" t="n">
-        <v>2025.0</v>
+        <v>2024.0</v>
       </c>
       <c r="F78" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="G78" t="s">
-        <v>82</v>
+        <v>199</v>
       </c>
       <c r="H78" t="s">
         <v>27</v>
@@ -7281,34 +7315,34 @@
         <v>70.0</v>
       </c>
       <c r="M78" t="n">
-        <v>220.0</v>
+        <v>190.0</v>
       </c>
       <c r="N78" t="s">
-        <v>453</v>
+        <v>462</v>
       </c>
       <c r="O78" t="n">
-        <v>12.0</v>
-      </c>
-      <c r="P78" t="s">
-        <v>454</v>
-      </c>
-      <c r="Q78" t="s">
-        <v>42</v>
+        <v>12.5</v>
+      </c>
+      <c r="P78" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>6.5</v>
       </c>
       <c r="R78" t="s">
         <v>32</v>
       </c>
       <c r="S78" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="T78" t="s">
-        <v>193</v>
+        <v>461</v>
       </c>
       <c r="U78" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
       <c r="V78" t="s">
-        <v>456</v>
+        <v>464</v>
       </c>
     </row>
     <row r="79">
@@ -7319,7 +7353,7 @@
         <v>78.0</v>
       </c>
       <c r="C79" t="s">
-        <v>193</v>
+        <v>465</v>
       </c>
       <c r="D79" t="s">
         <v>24</v>
@@ -7328,10 +7362,10 @@
         <v>2025.0</v>
       </c>
       <c r="F79" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="G79" t="s">
-        <v>48</v>
+        <v>154</v>
       </c>
       <c r="H79" t="s">
         <v>27</v>
@@ -7349,34 +7383,34 @@
         <v>70.0</v>
       </c>
       <c r="M79" t="n">
-        <v>199.0</v>
+        <v>197.0</v>
       </c>
       <c r="N79" t="s">
-        <v>457</v>
-      </c>
-      <c r="O79" t="n">
-        <v>11.0</v>
+        <v>466</v>
+      </c>
+      <c r="O79" t="s">
+        <v>112</v>
       </c>
       <c r="P79" t="s">
-        <v>31</v>
+        <v>172</v>
       </c>
       <c r="Q79" t="s">
-        <v>99</v>
+        <v>173</v>
       </c>
       <c r="R79" t="s">
         <v>32</v>
       </c>
       <c r="S79" t="s">
-        <v>43</v>
+        <v>75</v>
       </c>
       <c r="T79" t="s">
-        <v>193</v>
+        <v>465</v>
       </c>
       <c r="U79" t="s">
-        <v>458</v>
+        <v>467</v>
       </c>
       <c r="V79" t="s">
-        <v>459</v>
+        <v>468</v>
       </c>
     </row>
     <row r="80">
@@ -7387,13 +7421,13 @@
         <v>79.0</v>
       </c>
       <c r="C80" t="s">
-        <v>193</v>
+        <v>100</v>
       </c>
       <c r="D80" t="s">
         <v>24</v>
       </c>
       <c r="E80" t="n">
-        <v>2025.0</v>
+        <v>2024.0</v>
       </c>
       <c r="F80" t="s">
         <v>47</v>
@@ -7417,34 +7451,34 @@
         <v>70.0</v>
       </c>
       <c r="M80" t="n">
-        <v>250.0</v>
+        <v>280.0</v>
       </c>
       <c r="N80" t="s">
-        <v>460</v>
-      </c>
-      <c r="O80" t="n">
-        <v>12.0</v>
+        <v>469</v>
+      </c>
+      <c r="O80" t="s">
+        <v>242</v>
       </c>
       <c r="P80" t="s">
-        <v>113</v>
+        <v>71</v>
       </c>
       <c r="Q80" t="s">
-        <v>161</v>
+        <v>381</v>
       </c>
       <c r="R80" t="s">
         <v>32</v>
       </c>
       <c r="S80" t="s">
-        <v>43</v>
+        <v>100</v>
       </c>
       <c r="T80" t="s">
-        <v>193</v>
+        <v>100</v>
       </c>
       <c r="U80" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="V80" t="s">
-        <v>462</v>
+        <v>471</v>
       </c>
     </row>
     <row r="81">
@@ -7467,7 +7501,7 @@
         <v>47</v>
       </c>
       <c r="G81" t="s">
-        <v>148</v>
+        <v>48</v>
       </c>
       <c r="H81" t="s">
         <v>27</v>
@@ -7485,19 +7519,19 @@
         <v>70.0</v>
       </c>
       <c r="M81" t="n">
-        <v>220.0</v>
+        <v>199.0</v>
       </c>
       <c r="N81" t="s">
-        <v>463</v>
+        <v>472</v>
       </c>
       <c r="O81" t="n">
-        <v>12.0</v>
+        <v>11.0</v>
       </c>
       <c r="P81" t="s">
-        <v>447</v>
+        <v>31</v>
       </c>
       <c r="Q81" t="s">
-        <v>65</v>
+        <v>99</v>
       </c>
       <c r="R81" t="s">
         <v>32</v>
@@ -7509,10 +7543,10 @@
         <v>193</v>
       </c>
       <c r="U81" t="s">
-        <v>464</v>
+        <v>473</v>
       </c>
       <c r="V81" t="s">
-        <v>465</v>
+        <v>474</v>
       </c>
     </row>
     <row r="82">
@@ -7523,7 +7557,7 @@
         <v>81.0</v>
       </c>
       <c r="C82" t="s">
-        <v>100</v>
+        <v>193</v>
       </c>
       <c r="D82" t="s">
         <v>24</v>
@@ -7535,7 +7569,7 @@
         <v>47</v>
       </c>
       <c r="G82" t="s">
-        <v>82</v>
+        <v>148</v>
       </c>
       <c r="H82" t="s">
         <v>27</v>
@@ -7556,31 +7590,31 @@
         <v>220.0</v>
       </c>
       <c r="N82" t="s">
-        <v>466</v>
+        <v>475</v>
       </c>
       <c r="O82" t="n">
         <v>12.0</v>
       </c>
       <c r="P82" t="s">
-        <v>50</v>
+        <v>476</v>
       </c>
       <c r="Q82" t="s">
-        <v>447</v>
+        <v>65</v>
       </c>
       <c r="R82" t="s">
         <v>32</v>
       </c>
       <c r="S82" t="s">
-        <v>100</v>
+        <v>43</v>
       </c>
       <c r="T82" t="s">
-        <v>467</v>
+        <v>193</v>
       </c>
       <c r="U82" t="s">
-        <v>468</v>
+        <v>477</v>
       </c>
       <c r="V82" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
     </row>
     <row r="83">
@@ -7591,49 +7625,49 @@
         <v>82.0</v>
       </c>
       <c r="C83" t="s">
-        <v>204</v>
+        <v>479</v>
       </c>
       <c r="D83" t="s">
-        <v>24</v>
+        <v>220</v>
       </c>
       <c r="E83" t="n">
-        <v>2025.0</v>
+        <v>2024.0</v>
       </c>
       <c r="F83" t="s">
         <v>47</v>
       </c>
       <c r="G83" t="s">
-        <v>247</v>
+        <v>133</v>
       </c>
       <c r="H83" t="s">
         <v>27</v>
       </c>
       <c r="I83" t="n">
-        <v>19.0</v>
+        <v>16.0</v>
       </c>
       <c r="J83" t="n">
-        <v>42.0</v>
+        <v>36.0</v>
       </c>
       <c r="K83" t="n">
-        <v>65.0</v>
+        <v>57.0</v>
       </c>
       <c r="L83" t="n">
         <v>70.0</v>
       </c>
       <c r="M83" t="n">
-        <v>240.0</v>
+        <v>205.0</v>
       </c>
       <c r="N83" t="s">
-        <v>470</v>
-      </c>
-      <c r="O83" t="s">
-        <v>78</v>
-      </c>
-      <c r="P83" t="s">
-        <v>471</v>
-      </c>
-      <c r="Q83" t="s">
-        <v>232</v>
+        <v>480</v>
+      </c>
+      <c r="O83" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P83" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>6.9</v>
       </c>
       <c r="R83" t="s">
         <v>32</v>
@@ -7642,13 +7676,13 @@
         <v>100</v>
       </c>
       <c r="T83" t="s">
-        <v>204</v>
+        <v>479</v>
       </c>
       <c r="U83" t="s">
-        <v>472</v>
+        <v>481</v>
       </c>
       <c r="V83" t="s">
-        <v>473</v>
+        <v>482</v>
       </c>
     </row>
     <row r="84">
@@ -7659,64 +7693,64 @@
         <v>83.0</v>
       </c>
       <c r="C84" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="D84" t="s">
-        <v>24</v>
+        <v>283</v>
       </c>
       <c r="E84" t="n">
-        <v>2025.0</v>
+        <v>2021.0</v>
       </c>
       <c r="F84" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="G84" t="s">
-        <v>96</v>
+        <v>483</v>
       </c>
       <c r="H84" t="s">
-        <v>27</v>
+        <v>351</v>
       </c>
       <c r="I84" t="n">
-        <v>16.0</v>
+        <v>22.0</v>
       </c>
       <c r="J84" t="n">
-        <v>36.0</v>
+        <v>43.0</v>
       </c>
       <c r="K84" t="n">
-        <v>57.0</v>
+        <v>71.0</v>
       </c>
       <c r="L84" t="n">
         <v>70.0</v>
       </c>
       <c r="M84" t="n">
-        <v>190.0</v>
+        <v>160.0</v>
       </c>
       <c r="N84" t="s">
-        <v>474</v>
+        <v>484</v>
       </c>
       <c r="O84" t="s">
         <v>78</v>
       </c>
       <c r="P84" t="s">
-        <v>173</v>
+        <v>485</v>
       </c>
       <c r="Q84" t="s">
-        <v>79</v>
+        <v>206</v>
       </c>
       <c r="R84" t="s">
         <v>32</v>
       </c>
       <c r="S84" t="s">
-        <v>100</v>
+        <v>218</v>
       </c>
       <c r="T84" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="U84" t="s">
-        <v>475</v>
+        <v>486</v>
       </c>
       <c r="V84" t="s">
-        <v>476</v>
+        <v>487</v>
       </c>
     </row>
     <row r="85">
@@ -7727,64 +7761,64 @@
         <v>84.0</v>
       </c>
       <c r="C85" t="s">
-        <v>204</v>
+        <v>292</v>
       </c>
       <c r="D85" t="s">
-        <v>220</v>
+        <v>283</v>
       </c>
       <c r="E85" t="n">
         <v>2025.0</v>
       </c>
       <c r="F85" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="G85" t="s">
-        <v>125</v>
+        <v>148</v>
       </c>
       <c r="H85" t="s">
         <v>27</v>
       </c>
       <c r="I85" t="n">
-        <v>16.0</v>
+        <v>19.0</v>
       </c>
       <c r="J85" t="n">
-        <v>36.0</v>
+        <v>42.0</v>
       </c>
       <c r="K85" t="n">
-        <v>57.0</v>
+        <v>65.0</v>
       </c>
       <c r="L85" t="n">
         <v>70.0</v>
       </c>
       <c r="M85" t="n">
-        <v>190.0</v>
+        <v>280.0</v>
       </c>
       <c r="N85" t="s">
-        <v>477</v>
-      </c>
-      <c r="O85" t="s">
-        <v>78</v>
+        <v>488</v>
+      </c>
+      <c r="O85" t="n">
+        <v>11.0</v>
       </c>
       <c r="P85" t="s">
-        <v>478</v>
+        <v>489</v>
       </c>
       <c r="Q85" t="s">
-        <v>166</v>
+        <v>114</v>
       </c>
       <c r="R85" t="s">
         <v>32</v>
       </c>
       <c r="S85" t="s">
-        <v>100</v>
+        <v>292</v>
       </c>
       <c r="T85" t="s">
-        <v>204</v>
+        <v>292</v>
       </c>
       <c r="U85" t="s">
-        <v>479</v>
+        <v>490</v>
       </c>
       <c r="V85" t="s">
-        <v>480</v>
+        <v>491</v>
       </c>
     </row>
     <row r="86">
@@ -7795,64 +7829,64 @@
         <v>85.0</v>
       </c>
       <c r="C86" t="s">
-        <v>204</v>
+        <v>292</v>
       </c>
       <c r="D86" t="s">
-        <v>220</v>
+        <v>329</v>
       </c>
       <c r="E86" t="n">
-        <v>2025.0</v>
+        <v>2022.0</v>
       </c>
       <c r="F86" t="s">
-        <v>47</v>
+        <v>341</v>
       </c>
       <c r="G86" t="s">
-        <v>158</v>
+        <v>483</v>
       </c>
       <c r="H86" t="s">
-        <v>27</v>
+        <v>351</v>
       </c>
       <c r="I86" t="n">
-        <v>16.0</v>
+        <v>22.0</v>
       </c>
       <c r="J86" t="n">
-        <v>36.0</v>
+        <v>43.0</v>
       </c>
       <c r="K86" t="n">
-        <v>57.0</v>
+        <v>71.0</v>
       </c>
       <c r="L86" t="n">
         <v>70.0</v>
       </c>
       <c r="M86" t="n">
-        <v>209.0</v>
+        <v>180.0</v>
       </c>
       <c r="N86" t="s">
-        <v>481</v>
-      </c>
-      <c r="O86" t="n">
-        <v>12.0</v>
+        <v>492</v>
+      </c>
+      <c r="O86" t="s">
+        <v>265</v>
       </c>
       <c r="P86" t="s">
-        <v>482</v>
+        <v>493</v>
       </c>
       <c r="Q86" t="s">
-        <v>172</v>
+        <v>494</v>
       </c>
       <c r="R86" t="s">
         <v>32</v>
       </c>
       <c r="S86" t="s">
-        <v>100</v>
+        <v>292</v>
       </c>
       <c r="T86" t="s">
-        <v>204</v>
+        <v>292</v>
       </c>
       <c r="U86" t="s">
-        <v>483</v>
+        <v>495</v>
       </c>
       <c r="V86" t="s">
-        <v>484</v>
+        <v>496</v>
       </c>
     </row>
     <row r="87">
@@ -7863,7 +7897,7 @@
         <v>86.0</v>
       </c>
       <c r="C87" t="s">
-        <v>485</v>
+        <v>497</v>
       </c>
       <c r="D87" t="s">
         <v>24</v>
@@ -7896,7 +7930,7 @@
         <v>290.0</v>
       </c>
       <c r="N87" t="s">
-        <v>486</v>
+        <v>498</v>
       </c>
       <c r="O87" t="n">
         <v>14.0</v>
@@ -7914,13 +7948,13 @@
         <v>106</v>
       </c>
       <c r="T87" t="s">
-        <v>485</v>
+        <v>497</v>
       </c>
       <c r="U87" t="s">
-        <v>487</v>
+        <v>499</v>
       </c>
       <c r="V87" t="s">
-        <v>488</v>
+        <v>500</v>
       </c>
     </row>
     <row r="88">
@@ -7931,7 +7965,7 @@
         <v>87.0</v>
       </c>
       <c r="C88" t="s">
-        <v>489</v>
+        <v>501</v>
       </c>
       <c r="D88" t="s">
         <v>24</v>
@@ -7964,13 +7998,13 @@
         <v>423.0</v>
       </c>
       <c r="N88" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="O88" t="s">
         <v>78</v>
       </c>
       <c r="P88" t="s">
-        <v>436</v>
+        <v>503</v>
       </c>
       <c r="Q88" t="s">
         <v>172</v>
@@ -7982,13 +8016,13 @@
         <v>33</v>
       </c>
       <c r="T88" t="s">
-        <v>489</v>
+        <v>501</v>
       </c>
       <c r="U88" t="s">
-        <v>491</v>
+        <v>504</v>
       </c>
       <c r="V88" t="s">
-        <v>492</v>
+        <v>505</v>
       </c>
     </row>
     <row r="89">
@@ -7999,7 +8033,7 @@
         <v>88.0</v>
       </c>
       <c r="C89" t="s">
-        <v>493</v>
+        <v>506</v>
       </c>
       <c r="D89" t="s">
         <v>24</v>
@@ -8011,7 +8045,7 @@
         <v>47</v>
       </c>
       <c r="G89" t="s">
-        <v>494</v>
+        <v>507</v>
       </c>
       <c r="H89" t="s">
         <v>27</v>
@@ -8032,7 +8066,7 @@
         <v>510.0</v>
       </c>
       <c r="N89" t="s">
-        <v>495</v>
+        <v>508</v>
       </c>
       <c r="O89" t="n">
         <v>13.0</v>
@@ -8050,13 +8084,13 @@
         <v>100</v>
       </c>
       <c r="T89" t="s">
-        <v>493</v>
+        <v>506</v>
       </c>
       <c r="U89" t="s">
-        <v>496</v>
+        <v>509</v>
       </c>
       <c r="V89" t="s">
-        <v>497</v>
+        <v>510</v>
       </c>
     </row>
     <row r="90">
@@ -8067,7 +8101,7 @@
         <v>89.0</v>
       </c>
       <c r="C90" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="D90" t="s">
         <v>24</v>
@@ -8079,7 +8113,7 @@
         <v>25</v>
       </c>
       <c r="G90" t="s">
-        <v>499</v>
+        <v>512</v>
       </c>
       <c r="H90" t="s">
         <v>27</v>
@@ -8100,7 +8134,7 @@
         <v>420.0</v>
       </c>
       <c r="N90" t="s">
-        <v>500</v>
+        <v>513</v>
       </c>
       <c r="O90" t="n">
         <v>14.0</v>
@@ -8109,7 +8143,7 @@
         <v>0.0</v>
       </c>
       <c r="Q90" t="s">
-        <v>501</v>
+        <v>448</v>
       </c>
       <c r="R90" t="s">
         <v>32</v>
@@ -8118,13 +8152,13 @@
         <v>218</v>
       </c>
       <c r="T90" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="U90" t="s">
-        <v>502</v>
+        <v>514</v>
       </c>
       <c r="V90" t="s">
-        <v>503</v>
+        <v>515</v>
       </c>
     </row>
     <row r="91">
@@ -8135,7 +8169,7 @@
         <v>90.0</v>
       </c>
       <c r="C91" t="s">
-        <v>504</v>
+        <v>516</v>
       </c>
       <c r="D91" t="s">
         <v>24</v>
@@ -8144,10 +8178,10 @@
         <v>2024.0</v>
       </c>
       <c r="F91" t="s">
-        <v>505</v>
+        <v>517</v>
       </c>
       <c r="G91" t="s">
-        <v>506</v>
+        <v>518</v>
       </c>
       <c r="H91" t="s">
         <v>27</v>
@@ -8168,13 +8202,13 @@
         <v>363.0</v>
       </c>
       <c r="N91" t="s">
-        <v>507</v>
+        <v>519</v>
       </c>
       <c r="O91" t="s">
         <v>237</v>
       </c>
       <c r="P91" t="s">
-        <v>508</v>
+        <v>520</v>
       </c>
       <c r="Q91" t="s">
         <v>286</v>
@@ -8186,13 +8220,13 @@
         <v>33</v>
       </c>
       <c r="T91" t="s">
-        <v>504</v>
+        <v>516</v>
       </c>
       <c r="U91" t="s">
-        <v>509</v>
+        <v>521</v>
       </c>
       <c r="V91" t="s">
-        <v>510</v>
+        <v>522</v>
       </c>
     </row>
     <row r="92">
@@ -8203,7 +8237,7 @@
         <v>91.0</v>
       </c>
       <c r="C92" t="s">
-        <v>511</v>
+        <v>523</v>
       </c>
       <c r="D92" t="s">
         <v>24</v>
@@ -8215,7 +8249,7 @@
         <v>25</v>
       </c>
       <c r="G92" t="s">
-        <v>512</v>
+        <v>524</v>
       </c>
       <c r="H92" t="s">
         <v>27</v>
@@ -8236,13 +8270,13 @@
         <v>295.0</v>
       </c>
       <c r="N92" t="s">
-        <v>513</v>
+        <v>525</v>
       </c>
       <c r="O92" t="n">
         <v>13.0</v>
       </c>
       <c r="P92" t="s">
-        <v>436</v>
+        <v>503</v>
       </c>
       <c r="Q92" t="s">
         <v>177</v>
@@ -8254,13 +8288,13 @@
         <v>100</v>
       </c>
       <c r="T92" t="s">
-        <v>511</v>
+        <v>523</v>
       </c>
       <c r="U92" t="s">
-        <v>514</v>
+        <v>526</v>
       </c>
       <c r="V92" t="s">
-        <v>515</v>
+        <v>527</v>
       </c>
     </row>
     <row r="93">
@@ -8283,7 +8317,7 @@
         <v>37</v>
       </c>
       <c r="G93" t="s">
-        <v>516</v>
+        <v>528</v>
       </c>
       <c r="H93" t="s">
         <v>27</v>
@@ -8304,7 +8338,7 @@
         <v>242.0</v>
       </c>
       <c r="N93" t="s">
-        <v>517</v>
+        <v>529</v>
       </c>
       <c r="O93" t="s">
         <v>29</v>
@@ -8325,10 +8359,10 @@
         <v>106</v>
       </c>
       <c r="U93" t="s">
-        <v>518</v>
+        <v>530</v>
       </c>
       <c r="V93" t="s">
-        <v>519</v>
+        <v>531</v>
       </c>
     </row>
     <row r="94">
@@ -8339,7 +8373,7 @@
         <v>93.0</v>
       </c>
       <c r="C94" t="s">
-        <v>520</v>
+        <v>532</v>
       </c>
       <c r="D94" t="s">
         <v>220</v>
@@ -8351,7 +8385,7 @@
         <v>25</v>
       </c>
       <c r="G94" t="s">
-        <v>521</v>
+        <v>533</v>
       </c>
       <c r="H94" t="s">
         <v>27</v>
@@ -8372,7 +8406,7 @@
         <v>220.0</v>
       </c>
       <c r="N94" t="s">
-        <v>522</v>
+        <v>534</v>
       </c>
       <c r="O94" t="s">
         <v>40</v>
@@ -8390,13 +8424,13 @@
         <v>397</v>
       </c>
       <c r="T94" t="s">
-        <v>520</v>
+        <v>532</v>
       </c>
       <c r="U94" t="s">
-        <v>523</v>
+        <v>535</v>
       </c>
       <c r="V94" t="s">
-        <v>524</v>
+        <v>536</v>
       </c>
     </row>
     <row r="95">
@@ -8419,7 +8453,7 @@
         <v>25</v>
       </c>
       <c r="G95" t="s">
-        <v>499</v>
+        <v>512</v>
       </c>
       <c r="H95" t="s">
         <v>27</v>
@@ -8440,7 +8474,7 @@
         <v>220.0</v>
       </c>
       <c r="N95" t="s">
-        <v>525</v>
+        <v>537</v>
       </c>
       <c r="O95" t="n">
         <v>12.0</v>
@@ -8461,10 +8495,10 @@
         <v>43</v>
       </c>
       <c r="U95" t="s">
-        <v>526</v>
+        <v>538</v>
       </c>
       <c r="V95" t="s">
-        <v>527</v>
+        <v>539</v>
       </c>
     </row>
     <row r="96">
@@ -8475,7 +8509,7 @@
         <v>95.0</v>
       </c>
       <c r="C96" t="s">
-        <v>528</v>
+        <v>540</v>
       </c>
       <c r="D96" t="s">
         <v>24</v>
@@ -8487,7 +8521,7 @@
         <v>25</v>
       </c>
       <c r="G96" t="s">
-        <v>529</v>
+        <v>541</v>
       </c>
       <c r="H96" t="s">
         <v>27</v>
@@ -8508,7 +8542,7 @@
         <v>350.0</v>
       </c>
       <c r="N96" t="s">
-        <v>530</v>
+        <v>542</v>
       </c>
       <c r="O96" t="n">
         <v>14.0</v>
@@ -8526,13 +8560,13 @@
         <v>43</v>
       </c>
       <c r="T96" t="s">
-        <v>528</v>
+        <v>540</v>
       </c>
       <c r="U96" t="s">
-        <v>531</v>
+        <v>543</v>
       </c>
       <c r="V96" t="s">
-        <v>532</v>
+        <v>544</v>
       </c>
     </row>
     <row r="97">
@@ -8555,7 +8589,7 @@
         <v>25</v>
       </c>
       <c r="G97" t="s">
-        <v>533</v>
+        <v>545</v>
       </c>
       <c r="H97" t="s">
         <v>27</v>
@@ -8576,16 +8610,16 @@
         <v>290.0</v>
       </c>
       <c r="N97" t="s">
-        <v>534</v>
+        <v>546</v>
       </c>
       <c r="O97" t="s">
         <v>112</v>
       </c>
       <c r="P97" t="s">
-        <v>535</v>
+        <v>547</v>
       </c>
       <c r="Q97" t="s">
-        <v>536</v>
+        <v>548</v>
       </c>
       <c r="R97" t="s">
         <v>32</v>
@@ -8597,10 +8631,10 @@
         <v>218</v>
       </c>
       <c r="U97" t="s">
-        <v>537</v>
+        <v>549</v>
       </c>
       <c r="V97" t="s">
-        <v>538</v>
+        <v>550</v>
       </c>
     </row>
     <row r="98">
@@ -8623,7 +8657,7 @@
         <v>25</v>
       </c>
       <c r="G98" t="s">
-        <v>539</v>
+        <v>551</v>
       </c>
       <c r="H98" t="s">
         <v>27</v>
@@ -8644,16 +8678,16 @@
         <v>239.0</v>
       </c>
       <c r="N98" t="s">
-        <v>540</v>
+        <v>552</v>
       </c>
       <c r="O98" t="s">
         <v>78</v>
       </c>
       <c r="P98" t="s">
-        <v>541</v>
+        <v>553</v>
       </c>
       <c r="Q98" t="s">
-        <v>447</v>
+        <v>476</v>
       </c>
       <c r="R98" t="s">
         <v>32</v>
@@ -8662,13 +8696,13 @@
         <v>75</v>
       </c>
       <c r="T98" t="s">
-        <v>542</v>
+        <v>554</v>
       </c>
       <c r="U98" t="s">
-        <v>543</v>
+        <v>555</v>
       </c>
       <c r="V98" t="s">
-        <v>544</v>
+        <v>556</v>
       </c>
     </row>
     <row r="99">
@@ -8679,7 +8713,7 @@
         <v>98.0</v>
       </c>
       <c r="C99" t="s">
-        <v>545</v>
+        <v>557</v>
       </c>
       <c r="D99" t="s">
         <v>283</v>
@@ -8691,7 +8725,7 @@
         <v>37</v>
       </c>
       <c r="G99" t="s">
-        <v>546</v>
+        <v>558</v>
       </c>
       <c r="H99" t="s">
         <v>27</v>
@@ -8712,13 +8746,13 @@
         <v>239.99</v>
       </c>
       <c r="N99" t="s">
-        <v>547</v>
+        <v>559</v>
       </c>
       <c r="O99" t="s">
         <v>40</v>
       </c>
       <c r="P99" t="s">
-        <v>548</v>
+        <v>560</v>
       </c>
       <c r="Q99" t="s">
         <v>166</v>
@@ -8730,13 +8764,13 @@
         <v>33</v>
       </c>
       <c r="T99" t="s">
-        <v>545</v>
+        <v>557</v>
       </c>
       <c r="U99" t="s">
-        <v>549</v>
+        <v>561</v>
       </c>
       <c r="V99" t="s">
-        <v>550</v>
+        <v>562</v>
       </c>
     </row>
     <row r="100">
@@ -8759,7 +8793,7 @@
         <v>25</v>
       </c>
       <c r="G100" t="s">
-        <v>551</v>
+        <v>563</v>
       </c>
       <c r="H100" t="s">
         <v>27</v>
@@ -8780,13 +8814,13 @@
         <v>180.0</v>
       </c>
       <c r="N100" t="s">
-        <v>552</v>
+        <v>564</v>
       </c>
       <c r="O100" t="n">
         <v>11.0</v>
       </c>
       <c r="P100" t="s">
-        <v>553</v>
+        <v>565</v>
       </c>
       <c r="Q100" t="s">
         <v>99</v>
@@ -8801,10 +8835,10 @@
         <v>311</v>
       </c>
       <c r="U100" t="s">
-        <v>554</v>
+        <v>566</v>
       </c>
       <c r="V100" t="s">
-        <v>555</v>
+        <v>567</v>
       </c>
     </row>
     <row r="101">
@@ -8827,7 +8861,7 @@
         <v>55</v>
       </c>
       <c r="G101" t="s">
-        <v>556</v>
+        <v>568</v>
       </c>
       <c r="H101" t="s">
         <v>27</v>
@@ -8848,7 +8882,7 @@
         <v>250.0</v>
       </c>
       <c r="N101" t="s">
-        <v>557</v>
+        <v>569</v>
       </c>
       <c r="O101" t="s">
         <v>265</v>
@@ -8866,13 +8900,13 @@
         <v>292</v>
       </c>
       <c r="T101" t="s">
-        <v>558</v>
+        <v>570</v>
       </c>
       <c r="U101" t="s">
-        <v>559</v>
+        <v>571</v>
       </c>
       <c r="V101" t="s">
-        <v>560</v>
+        <v>572</v>
       </c>
     </row>
     <row r="102">
@@ -8883,7 +8917,7 @@
         <v>101.0</v>
       </c>
       <c r="C102" t="s">
-        <v>561</v>
+        <v>573</v>
       </c>
       <c r="D102" t="s">
         <v>283</v>
@@ -8895,7 +8929,7 @@
         <v>25</v>
       </c>
       <c r="G102" t="s">
-        <v>562</v>
+        <v>483</v>
       </c>
       <c r="H102" t="s">
         <v>27</v>
@@ -8916,13 +8950,13 @@
         <v>130.0</v>
       </c>
       <c r="N102" t="s">
-        <v>563</v>
+        <v>574</v>
       </c>
       <c r="O102" t="n">
         <v>9.0</v>
       </c>
       <c r="P102" t="s">
-        <v>564</v>
+        <v>575</v>
       </c>
       <c r="Q102" t="s">
         <v>156</v>
@@ -8934,13 +8968,13 @@
         <v>226</v>
       </c>
       <c r="T102" t="s">
-        <v>561</v>
+        <v>573</v>
       </c>
       <c r="U102" t="s">
         <v>152</v>
       </c>
       <c r="V102" t="s">
-        <v>565</v>
+        <v>576</v>
       </c>
     </row>
     <row r="103">
@@ -8951,7 +8985,7 @@
         <v>102.0</v>
       </c>
       <c r="C103" t="s">
-        <v>566</v>
+        <v>577</v>
       </c>
       <c r="D103" t="s">
         <v>24</v>
@@ -8984,7 +9018,7 @@
         <v>119.0</v>
       </c>
       <c r="N103" t="s">
-        <v>567</v>
+        <v>578</v>
       </c>
       <c r="O103" t="n">
         <v>12.5</v>
@@ -9002,13 +9036,13 @@
         <v>191</v>
       </c>
       <c r="T103" t="s">
-        <v>566</v>
+        <v>577</v>
       </c>
       <c r="U103" t="s">
-        <v>568</v>
+        <v>579</v>
       </c>
       <c r="V103" t="s">
-        <v>569</v>
+        <v>580</v>
       </c>
     </row>
     <row r="104">
@@ -9019,7 +9053,7 @@
         <v>103.0</v>
       </c>
       <c r="C104" t="s">
-        <v>570</v>
+        <v>581</v>
       </c>
       <c r="D104" t="s">
         <v>24</v>
@@ -9052,13 +9086,13 @@
         <v>230.0</v>
       </c>
       <c r="N104" t="s">
-        <v>571</v>
+        <v>582</v>
       </c>
       <c r="O104" t="s">
         <v>40</v>
       </c>
       <c r="P104" t="s">
-        <v>572</v>
+        <v>583</v>
       </c>
       <c r="Q104" t="s">
         <v>156</v>
@@ -9070,13 +9104,13 @@
         <v>51</v>
       </c>
       <c r="T104" t="s">
-        <v>570</v>
+        <v>581</v>
       </c>
       <c r="U104" t="s">
-        <v>573</v>
+        <v>584</v>
       </c>
       <c r="V104" t="s">
-        <v>574</v>
+        <v>585</v>
       </c>
     </row>
     <row r="105">
@@ -9087,7 +9121,7 @@
         <v>104.0</v>
       </c>
       <c r="C105" t="s">
-        <v>575</v>
+        <v>586</v>
       </c>
       <c r="D105" t="s">
         <v>283</v>
@@ -9120,7 +9154,7 @@
         <v>195.0</v>
       </c>
       <c r="N105" t="s">
-        <v>576</v>
+        <v>587</v>
       </c>
       <c r="O105" t="n">
         <v>11.5</v>
@@ -9135,16 +9169,16 @@
         <v>32</v>
       </c>
       <c r="S105" t="s">
-        <v>577</v>
+        <v>588</v>
       </c>
       <c r="T105" t="s">
-        <v>575</v>
+        <v>586</v>
       </c>
       <c r="U105" t="s">
-        <v>578</v>
+        <v>589</v>
       </c>
       <c r="V105" t="s">
-        <v>579</v>
+        <v>590</v>
       </c>
     </row>
     <row r="106">
@@ -9167,7 +9201,7 @@
         <v>25</v>
       </c>
       <c r="G106" t="s">
-        <v>580</v>
+        <v>591</v>
       </c>
       <c r="H106" t="s">
         <v>27</v>
@@ -9188,7 +9222,7 @@
         <v>295.0</v>
       </c>
       <c r="N106" t="s">
-        <v>581</v>
+        <v>592</v>
       </c>
       <c r="O106" t="s">
         <v>29</v>
@@ -9209,10 +9243,10 @@
         <v>58</v>
       </c>
       <c r="U106" t="s">
-        <v>582</v>
+        <v>593</v>
       </c>
       <c r="V106" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
     </row>
     <row r="107">
@@ -9256,16 +9290,16 @@
         <v>280.0</v>
       </c>
       <c r="N107" t="s">
-        <v>584</v>
+        <v>595</v>
       </c>
       <c r="O107" t="s">
         <v>78</v>
       </c>
       <c r="P107" t="s">
-        <v>585</v>
+        <v>596</v>
       </c>
       <c r="Q107" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="R107" t="s">
         <v>32</v>
@@ -9277,10 +9311,10 @@
         <v>193</v>
       </c>
       <c r="U107" t="s">
-        <v>587</v>
+        <v>598</v>
       </c>
       <c r="V107" t="s">
-        <v>588</v>
+        <v>599</v>
       </c>
     </row>
     <row r="108">
@@ -9291,7 +9325,7 @@
         <v>107.0</v>
       </c>
       <c r="C108" t="s">
-        <v>589</v>
+        <v>600</v>
       </c>
       <c r="D108" t="s">
         <v>24</v>
@@ -9324,7 +9358,7 @@
         <v>195.0</v>
       </c>
       <c r="N108" t="s">
-        <v>590</v>
+        <v>601</v>
       </c>
       <c r="O108" t="s">
         <v>112</v>
@@ -9333,7 +9367,7 @@
         <v>156</v>
       </c>
       <c r="Q108" t="s">
-        <v>501</v>
+        <v>448</v>
       </c>
       <c r="R108" t="s">
         <v>32</v>
@@ -9342,13 +9376,13 @@
         <v>218</v>
       </c>
       <c r="T108" t="s">
-        <v>589</v>
+        <v>600</v>
       </c>
       <c r="U108" t="s">
         <v>152</v>
       </c>
       <c r="V108" t="s">
-        <v>591</v>
+        <v>602</v>
       </c>
     </row>
     <row r="109">
@@ -9359,7 +9393,7 @@
         <v>108.0</v>
       </c>
       <c r="C109" t="s">
-        <v>592</v>
+        <v>603</v>
       </c>
       <c r="D109" t="s">
         <v>220</v>
@@ -9392,13 +9426,13 @@
         <v>180.0</v>
       </c>
       <c r="N109" t="s">
-        <v>593</v>
+        <v>604</v>
       </c>
       <c r="O109" t="n">
         <v>12.0</v>
       </c>
       <c r="P109" t="s">
-        <v>594</v>
+        <v>605</v>
       </c>
       <c r="Q109" t="n">
         <v>6.0</v>
@@ -9410,13 +9444,13 @@
         <v>33</v>
       </c>
       <c r="T109" t="s">
-        <v>592</v>
+        <v>603</v>
       </c>
       <c r="U109" t="s">
-        <v>595</v>
+        <v>606</v>
       </c>
       <c r="V109" t="s">
-        <v>596</v>
+        <v>607</v>
       </c>
     </row>
     <row r="110">
@@ -9427,7 +9461,7 @@
         <v>109.0</v>
       </c>
       <c r="C110" t="s">
-        <v>597</v>
+        <v>608</v>
       </c>
       <c r="D110" t="s">
         <v>283</v>
@@ -9460,7 +9494,7 @@
         <v>230.0</v>
       </c>
       <c r="N110" t="s">
-        <v>598</v>
+        <v>609</v>
       </c>
       <c r="O110" t="n">
         <v>12.5</v>
@@ -9478,13 +9512,13 @@
         <v>92</v>
       </c>
       <c r="T110" t="s">
-        <v>597</v>
+        <v>608</v>
       </c>
       <c r="U110" t="s">
-        <v>599</v>
+        <v>610</v>
       </c>
       <c r="V110" t="s">
-        <v>600</v>
+        <v>611</v>
       </c>
     </row>
     <row r="111">
@@ -9495,7 +9529,7 @@
         <v>110.0</v>
       </c>
       <c r="C111" t="s">
-        <v>601</v>
+        <v>612</v>
       </c>
       <c r="D111" t="s">
         <v>24</v>
@@ -9507,7 +9541,7 @@
         <v>37</v>
       </c>
       <c r="G111" t="s">
-        <v>602</v>
+        <v>613</v>
       </c>
       <c r="H111" t="s">
         <v>27</v>
@@ -9528,13 +9562,13 @@
         <v>209.0</v>
       </c>
       <c r="N111" t="s">
-        <v>603</v>
+        <v>614</v>
       </c>
       <c r="O111" t="n">
         <v>13.0</v>
       </c>
       <c r="P111" t="s">
-        <v>604</v>
+        <v>615</v>
       </c>
       <c r="Q111" t="s">
         <v>65</v>
@@ -9546,13 +9580,13 @@
         <v>51</v>
       </c>
       <c r="T111" t="s">
-        <v>601</v>
+        <v>612</v>
       </c>
       <c r="U111" t="s">
         <v>152</v>
       </c>
       <c r="V111" t="s">
-        <v>605</v>
+        <v>616</v>
       </c>
     </row>
     <row r="112">
@@ -9596,7 +9630,7 @@
         <v>240.0</v>
       </c>
       <c r="N112" t="s">
-        <v>606</v>
+        <v>617</v>
       </c>
       <c r="O112" t="n">
         <v>13.0</v>
@@ -9617,10 +9651,10 @@
         <v>292</v>
       </c>
       <c r="U112" t="s">
-        <v>607</v>
+        <v>618</v>
       </c>
       <c r="V112" t="s">
-        <v>608</v>
+        <v>619</v>
       </c>
     </row>
     <row r="113">
@@ -9631,7 +9665,7 @@
         <v>112.0</v>
       </c>
       <c r="C113" t="s">
-        <v>609</v>
+        <v>620</v>
       </c>
       <c r="D113" t="s">
         <v>24</v>
@@ -9664,7 +9698,7 @@
         <v>192.99</v>
       </c>
       <c r="N113" t="s">
-        <v>610</v>
+        <v>621</v>
       </c>
       <c r="O113" t="s">
         <v>90</v>
@@ -9682,13 +9716,13 @@
         <v>311</v>
       </c>
       <c r="T113" t="s">
-        <v>611</v>
+        <v>622</v>
       </c>
       <c r="U113" t="s">
-        <v>612</v>
+        <v>623</v>
       </c>
       <c r="V113" t="s">
-        <v>613</v>
+        <v>624</v>
       </c>
     </row>
     <row r="114">
@@ -9732,7 +9766,7 @@
         <v>189.0</v>
       </c>
       <c r="N114" t="s">
-        <v>614</v>
+        <v>625</v>
       </c>
       <c r="O114" t="n">
         <v>12.0</v>
@@ -9753,10 +9787,10 @@
         <v>204</v>
       </c>
       <c r="U114" t="s">
-        <v>615</v>
+        <v>626</v>
       </c>
       <c r="V114" t="s">
-        <v>616</v>
+        <v>627</v>
       </c>
     </row>
     <row r="115">
@@ -9767,7 +9801,7 @@
         <v>114.0</v>
       </c>
       <c r="C115" t="s">
-        <v>617</v>
+        <v>628</v>
       </c>
       <c r="D115" t="s">
         <v>220</v>
@@ -9800,7 +9834,7 @@
         <v>175.0</v>
       </c>
       <c r="N115" t="s">
-        <v>618</v>
+        <v>629</v>
       </c>
       <c r="O115" t="s">
         <v>242</v>
@@ -9818,13 +9852,13 @@
         <v>33</v>
       </c>
       <c r="T115" t="s">
-        <v>617</v>
+        <v>628</v>
       </c>
       <c r="U115" t="s">
-        <v>619</v>
+        <v>630</v>
       </c>
       <c r="V115" t="s">
-        <v>620</v>
+        <v>631</v>
       </c>
     </row>
     <row r="116">
@@ -9835,7 +9869,7 @@
         <v>115.0</v>
       </c>
       <c r="C116" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="D116" t="s">
         <v>220</v>
@@ -9847,7 +9881,7 @@
         <v>25</v>
       </c>
       <c r="G116" t="s">
-        <v>562</v>
+        <v>483</v>
       </c>
       <c r="H116" t="s">
         <v>27</v>
@@ -9868,13 +9902,13 @@
         <v>99.0</v>
       </c>
       <c r="N116" t="s">
-        <v>622</v>
+        <v>633</v>
       </c>
       <c r="O116" t="s">
         <v>265</v>
       </c>
       <c r="P116" t="s">
-        <v>623</v>
+        <v>634</v>
       </c>
       <c r="Q116" t="s">
         <v>232</v>
@@ -9883,16 +9917,16 @@
         <v>374</v>
       </c>
       <c r="S116" t="s">
-        <v>624</v>
+        <v>635</v>
       </c>
       <c r="T116" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="U116" t="s">
-        <v>625</v>
+        <v>636</v>
       </c>
       <c r="V116" t="s">
-        <v>626</v>
+        <v>637</v>
       </c>
     </row>
     <row r="117">
@@ -9903,7 +9937,7 @@
         <v>116.0</v>
       </c>
       <c r="C117" t="s">
-        <v>627</v>
+        <v>638</v>
       </c>
       <c r="D117" t="s">
         <v>24</v>
@@ -9915,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="G117" t="s">
-        <v>562</v>
+        <v>483</v>
       </c>
       <c r="H117" t="s">
         <v>27</v>
@@ -9936,7 +9970,7 @@
         <v>99.0</v>
       </c>
       <c r="N117" t="s">
-        <v>628</v>
+        <v>639</v>
       </c>
       <c r="O117" t="s">
         <v>40</v>
@@ -9954,13 +9988,13 @@
         <v>43</v>
       </c>
       <c r="T117" t="s">
-        <v>627</v>
+        <v>638</v>
       </c>
       <c r="U117" t="s">
-        <v>629</v>
+        <v>640</v>
       </c>
       <c r="V117" t="s">
-        <v>630</v>
+        <v>641</v>
       </c>
     </row>
     <row r="118">
@@ -9971,7 +10005,7 @@
         <v>117.0</v>
       </c>
       <c r="C118" t="s">
-        <v>631</v>
+        <v>642</v>
       </c>
       <c r="D118" t="s">
         <v>220</v>
@@ -10004,7 +10038,7 @@
         <v>140.0</v>
       </c>
       <c r="N118" t="s">
-        <v>632</v>
+        <v>643</v>
       </c>
       <c r="O118" t="n">
         <v>11.0</v>
@@ -10019,16 +10053,16 @@
         <v>374</v>
       </c>
       <c r="S118" t="s">
-        <v>633</v>
+        <v>644</v>
       </c>
       <c r="T118" t="s">
-        <v>631</v>
+        <v>642</v>
       </c>
       <c r="U118" t="s">
-        <v>634</v>
+        <v>645</v>
       </c>
       <c r="V118" t="s">
-        <v>635</v>
+        <v>646</v>
       </c>
     </row>
     <row r="119">
@@ -10039,7 +10073,7 @@
         <v>118.0</v>
       </c>
       <c r="C119" t="s">
-        <v>636</v>
+        <v>647</v>
       </c>
       <c r="D119" t="s">
         <v>283</v>
@@ -10072,7 +10106,7 @@
         <v>130.0</v>
       </c>
       <c r="N119" t="s">
-        <v>637</v>
+        <v>648</v>
       </c>
       <c r="O119" t="n">
         <v>10.0</v>
@@ -10090,13 +10124,13 @@
         <v>75</v>
       </c>
       <c r="T119" t="s">
-        <v>636</v>
+        <v>647</v>
       </c>
       <c r="U119" t="s">
-        <v>638</v>
+        <v>649</v>
       </c>
       <c r="V119" t="s">
-        <v>639</v>
+        <v>650</v>
       </c>
     </row>
     <row r="120">
@@ -10107,7 +10141,7 @@
         <v>119.0</v>
       </c>
       <c r="C120" t="s">
-        <v>640</v>
+        <v>651</v>
       </c>
       <c r="D120" t="s">
         <v>283</v>
@@ -10140,7 +10174,7 @@
         <v>140.0</v>
       </c>
       <c r="N120" t="s">
-        <v>641</v>
+        <v>652</v>
       </c>
       <c r="O120" t="n">
         <v>10.0</v>
@@ -10155,16 +10189,16 @@
         <v>374</v>
       </c>
       <c r="S120" t="s">
-        <v>624</v>
+        <v>635</v>
       </c>
       <c r="T120" t="s">
-        <v>640</v>
+        <v>651</v>
       </c>
       <c r="U120" t="s">
-        <v>642</v>
+        <v>653</v>
       </c>
       <c r="V120" t="s">
-        <v>643</v>
+        <v>654</v>
       </c>
     </row>
     <row r="121">
@@ -10175,7 +10209,7 @@
         <v>120.0</v>
       </c>
       <c r="C121" t="s">
-        <v>644</v>
+        <v>655</v>
       </c>
       <c r="D121" t="s">
         <v>220</v>
@@ -10208,7 +10242,7 @@
         <v>130.0</v>
       </c>
       <c r="N121" t="s">
-        <v>645</v>
+        <v>656</v>
       </c>
       <c r="O121" t="n">
         <v>11.0</v>
@@ -10226,13 +10260,13 @@
         <v>191</v>
       </c>
       <c r="T121" t="s">
-        <v>644</v>
+        <v>655</v>
       </c>
       <c r="U121" t="s">
-        <v>646</v>
+        <v>657</v>
       </c>
       <c r="V121" t="s">
-        <v>647</v>
+        <v>658</v>
       </c>
     </row>
   </sheetData>

</xml_diff>